<commit_message>
xong jk 1 jg1
</commit_message>
<xml_diff>
--- a/JK1/BAS-JK1 T7.xlsx
+++ b/JK1/BAS-JK1 T7.xlsx
@@ -1204,31 +1204,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1239,6 +1224,21 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2088,6 +2088,272 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10" descr="AUTO_FIT_CELL_PICTURE=K4"/>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21907501" y="1885950"/>
+          <a:ext cx="3209925" cy="1905000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 13" descr="AUTO_FIT_CELL_PICTURE=K5"/>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21907500" y="3790950"/>
+          <a:ext cx="3209925" cy="1905000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="Picture 18" descr="AUTO_FIT_CELL_PICTURE=K7"/>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21907501" y="7600950"/>
+          <a:ext cx="3209925" cy="1905000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Picture 19" descr="AUTO_FIT_CELL_PICTURE=K8"/>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21907501" y="9505950"/>
+          <a:ext cx="3209925" cy="1905000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Picture 20" descr="AUTO_FIT_CELL_PICTURE=K6"/>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21907500" y="5695950"/>
+          <a:ext cx="3209925" cy="1905000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="Picture 21" descr="AUTO_FIT_CELL_PICTURE=K9"/>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21907501" y="11410950"/>
+          <a:ext cx="3209925" cy="1905000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Picture 22" descr="AUTO_FIT_CELL_PICTURE=K10"/>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21907501" y="13315950"/>
+          <a:ext cx="3209925" cy="1905000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2562,22 +2828,22 @@
       <c r="Z4" s="23"/>
     </row>
     <row r="5" spans="1:26" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="61" t="s">
+      <c r="A5" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="63" t="s">
+      <c r="B5" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="63" t="s">
+      <c r="C5" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="64" t="s">
+      <c r="D5" s="69" t="s">
         <v>23</v>
       </c>
       <c r="E5" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="65" t="s">
+      <c r="F5" s="71" t="s">
         <v>25</v>
       </c>
       <c r="G5" s="24">
@@ -2616,14 +2882,14 @@
       <c r="Z5" s="23"/>
     </row>
     <row r="6" spans="1:26" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="62"/>
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
+      <c r="A6" s="61"/>
+      <c r="B6" s="61"/>
+      <c r="C6" s="61"/>
+      <c r="D6" s="61"/>
       <c r="E6" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="62"/>
+      <c r="F6" s="61"/>
       <c r="G6" s="26">
         <v>2</v>
       </c>
@@ -2637,7 +2903,7 @@
         <v>237</v>
       </c>
       <c r="K6" s="18"/>
-      <c r="L6" s="62"/>
+      <c r="L6" s="61"/>
       <c r="M6" s="20"/>
       <c r="N6" s="21"/>
       <c r="O6" s="22" t="s">
@@ -2714,22 +2980,22 @@
       <c r="Z7" s="23"/>
     </row>
     <row r="8" spans="1:26" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="63" t="s">
+      <c r="A8" s="68" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="63" t="s">
+      <c r="B8" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="63" t="s">
+      <c r="C8" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="64" t="s">
+      <c r="D8" s="69" t="s">
         <v>42</v>
       </c>
       <c r="E8" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="F8" s="66" t="s">
+      <c r="F8" s="72" t="s">
         <v>25</v>
       </c>
       <c r="G8" s="17">
@@ -2819,7 +3085,7 @@
       <c r="E10" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="62"/>
+      <c r="F10" s="61"/>
       <c r="G10" s="17">
         <v>3</v>
       </c>
@@ -3119,22 +3385,22 @@
       <c r="S17" s="27"/>
     </row>
     <row r="18" spans="1:26" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="63" t="s">
+      <c r="A18" s="68" t="s">
         <v>70</v>
       </c>
-      <c r="B18" s="63" t="s">
+      <c r="B18" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="63" t="s">
+      <c r="C18" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="65" t="s">
+      <c r="D18" s="71" t="s">
         <v>71</v>
       </c>
       <c r="E18" s="44" t="s">
         <v>72</v>
       </c>
-      <c r="F18" s="66" t="s">
+      <c r="F18" s="72" t="s">
         <v>25</v>
       </c>
       <c r="G18" s="45">
@@ -3255,14 +3521,14 @@
       <c r="Z20" s="48"/>
     </row>
     <row r="21" spans="1:26" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="62"/>
-      <c r="B21" s="62"/>
-      <c r="C21" s="62"/>
+      <c r="A21" s="61"/>
+      <c r="B21" s="61"/>
+      <c r="C21" s="61"/>
       <c r="D21" s="60"/>
       <c r="E21" s="44" t="s">
         <v>77</v>
       </c>
-      <c r="F21" s="62"/>
+      <c r="F21" s="61"/>
       <c r="G21" s="45">
         <v>4</v>
       </c>
@@ -3274,7 +3540,7 @@
       </c>
       <c r="J21" s="22"/>
       <c r="K21" s="18"/>
-      <c r="L21" s="62"/>
+      <c r="L21" s="61"/>
       <c r="M21" s="46"/>
       <c r="N21" s="47"/>
       <c r="O21" s="22" t="s">
@@ -3297,22 +3563,22 @@
       <c r="Z21" s="48"/>
     </row>
     <row r="22" spans="1:26" ht="16.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="63" t="s">
+      <c r="A22" s="68" t="s">
         <v>78</v>
       </c>
-      <c r="B22" s="63" t="s">
+      <c r="B22" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="63" t="s">
+      <c r="C22" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="D22" s="65" t="s">
+      <c r="D22" s="71" t="s">
         <v>79</v>
       </c>
       <c r="E22" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="F22" s="67" t="s">
+      <c r="F22" s="64" t="s">
         <v>25</v>
       </c>
       <c r="G22" s="17">
@@ -3517,14 +3783,14 @@
       <c r="Z26" s="23"/>
     </row>
     <row r="27" spans="1:26" ht="16.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="62"/>
-      <c r="B27" s="62"/>
-      <c r="C27" s="62"/>
-      <c r="D27" s="62"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
+      <c r="C27" s="61"/>
+      <c r="D27" s="61"/>
       <c r="E27" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="F27" s="62"/>
+      <c r="F27" s="61"/>
       <c r="G27" s="17">
         <v>6</v>
       </c>
@@ -3536,7 +3802,7 @@
       </c>
       <c r="J27" s="18"/>
       <c r="K27" s="18"/>
-      <c r="L27" s="62"/>
+      <c r="L27" s="61"/>
       <c r="M27" s="20"/>
       <c r="N27" s="21"/>
       <c r="O27" s="22" t="s">
@@ -3823,16 +4089,16 @@
       <c r="Z32" s="53"/>
     </row>
     <row r="33" spans="1:26" ht="16.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="61" t="s">
+      <c r="A33" s="63" t="s">
         <v>130</v>
       </c>
-      <c r="B33" s="63" t="s">
+      <c r="B33" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="C33" s="63" t="s">
+      <c r="C33" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="D33" s="64" t="s">
+      <c r="D33" s="69" t="s">
         <v>99</v>
       </c>
       <c r="E33" s="41" t="s">
@@ -3875,10 +4141,10 @@
       <c r="Z33" s="23"/>
     </row>
     <row r="34" spans="1:26" ht="16.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="62"/>
-      <c r="B34" s="62"/>
-      <c r="C34" s="62"/>
-      <c r="D34" s="62"/>
+      <c r="A34" s="61"/>
+      <c r="B34" s="61"/>
+      <c r="C34" s="61"/>
+      <c r="D34" s="61"/>
       <c r="E34" s="41" t="s">
         <v>136</v>
       </c>
@@ -3896,7 +4162,7 @@
       </c>
       <c r="J34" s="18"/>
       <c r="K34" s="18"/>
-      <c r="L34" s="62"/>
+      <c r="L34" s="61"/>
       <c r="M34" s="20"/>
       <c r="N34" s="21"/>
       <c r="O34" s="22" t="s">
@@ -4179,22 +4445,22 @@
       <c r="Z39" s="23"/>
     </row>
     <row r="40" spans="1:26" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="61" t="s">
+      <c r="A40" s="63" t="s">
         <v>170</v>
       </c>
-      <c r="B40" s="63" t="s">
+      <c r="B40" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="C40" s="63" t="s">
+      <c r="C40" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="D40" s="64" t="s">
+      <c r="D40" s="69" t="s">
         <v>171</v>
       </c>
-      <c r="E40" s="68" t="s">
+      <c r="E40" s="70" t="s">
         <v>172</v>
       </c>
-      <c r="F40" s="67" t="s">
+      <c r="F40" s="64" t="s">
         <v>25</v>
       </c>
       <c r="G40" s="24">
@@ -4274,11 +4540,11 @@
     </row>
     <row r="42" spans="1:26" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="60"/>
-      <c r="B42" s="62"/>
-      <c r="C42" s="62"/>
-      <c r="D42" s="62"/>
-      <c r="E42" s="62"/>
-      <c r="F42" s="62"/>
+      <c r="B42" s="61"/>
+      <c r="C42" s="61"/>
+      <c r="D42" s="61"/>
+      <c r="E42" s="61"/>
+      <c r="F42" s="61"/>
       <c r="G42" s="24">
         <v>3</v>
       </c>
@@ -4315,22 +4581,22 @@
       <c r="Z42" s="56"/>
     </row>
     <row r="43" spans="1:26" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="61" t="s">
+      <c r="A43" s="63" t="s">
         <v>181</v>
       </c>
-      <c r="B43" s="63" t="s">
+      <c r="B43" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="C43" s="63" t="s">
+      <c r="C43" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="D43" s="64" t="s">
+      <c r="D43" s="69" t="s">
         <v>171</v>
       </c>
-      <c r="E43" s="67" t="s">
+      <c r="E43" s="64" t="s">
         <v>182</v>
       </c>
-      <c r="F43" s="67" t="s">
+      <c r="F43" s="64" t="s">
         <v>25</v>
       </c>
       <c r="G43" s="24">
@@ -4409,12 +4675,12 @@
       <c r="Z44" s="56"/>
     </row>
     <row r="45" spans="1:26" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="62"/>
-      <c r="B45" s="62"/>
-      <c r="C45" s="62"/>
-      <c r="D45" s="62"/>
-      <c r="E45" s="62"/>
-      <c r="F45" s="62"/>
+      <c r="A45" s="61"/>
+      <c r="B45" s="61"/>
+      <c r="C45" s="61"/>
+      <c r="D45" s="61"/>
+      <c r="E45" s="61"/>
+      <c r="F45" s="61"/>
       <c r="G45" s="24">
         <v>3</v>
       </c>
@@ -4428,7 +4694,7 @@
         <v>237</v>
       </c>
       <c r="K45" s="18"/>
-      <c r="L45" s="62"/>
+      <c r="L45" s="61"/>
       <c r="M45" s="20"/>
       <c r="N45" s="21"/>
       <c r="O45" s="22" t="s">
@@ -4505,22 +4771,22 @@
       <c r="Z46" s="56"/>
     </row>
     <row r="47" spans="1:26" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="61" t="s">
+      <c r="A47" s="63" t="s">
         <v>189</v>
       </c>
-      <c r="B47" s="63" t="s">
+      <c r="B47" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="C47" s="63" t="s">
+      <c r="C47" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="D47" s="64" t="s">
+      <c r="D47" s="69" t="s">
         <v>190</v>
       </c>
-      <c r="E47" s="67" t="s">
+      <c r="E47" s="64" t="s">
         <v>191</v>
       </c>
-      <c r="F47" s="67" t="s">
+      <c r="F47" s="64" t="s">
         <v>25</v>
       </c>
       <c r="G47" s="24">
@@ -4560,9 +4826,9 @@
     </row>
     <row r="48" spans="1:26" ht="56.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="60"/>
-      <c r="B48" s="62"/>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
+      <c r="B48" s="61"/>
+      <c r="C48" s="61"/>
+      <c r="D48" s="61"/>
       <c r="E48" s="60"/>
       <c r="F48" s="60"/>
       <c r="G48" s="24">
@@ -4599,22 +4865,22 @@
       <c r="Z48" s="56"/>
     </row>
     <row r="49" spans="1:26" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="61" t="s">
+      <c r="A49" s="63" t="s">
         <v>196</v>
       </c>
-      <c r="B49" s="63" t="s">
+      <c r="B49" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="C49" s="63" t="s">
+      <c r="C49" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="D49" s="64" t="s">
+      <c r="D49" s="69" t="s">
         <v>190</v>
       </c>
-      <c r="E49" s="67" t="s">
+      <c r="E49" s="64" t="s">
         <v>197</v>
       </c>
-      <c r="F49" s="67" t="s">
+      <c r="F49" s="64" t="s">
         <v>25</v>
       </c>
       <c r="G49" s="24">
@@ -4653,10 +4919,10 @@
       <c r="Z49" s="56"/>
     </row>
     <row r="50" spans="1:26" ht="55.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="62"/>
-      <c r="B50" s="62"/>
-      <c r="C50" s="62"/>
-      <c r="D50" s="62"/>
+      <c r="A50" s="61"/>
+      <c r="B50" s="61"/>
+      <c r="C50" s="61"/>
+      <c r="D50" s="61"/>
       <c r="E50" s="60"/>
       <c r="F50" s="60"/>
       <c r="G50" s="24">
@@ -4670,7 +4936,7 @@
       </c>
       <c r="J50" s="18"/>
       <c r="K50" s="18"/>
-      <c r="L50" s="62"/>
+      <c r="L50" s="61"/>
       <c r="M50" s="20"/>
       <c r="N50" s="21"/>
       <c r="O50" s="22" t="s">
@@ -4747,22 +5013,22 @@
       <c r="Z51" s="56"/>
     </row>
     <row r="52" spans="1:26" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="61" t="s">
+      <c r="A52" s="63" t="s">
         <v>203</v>
       </c>
-      <c r="B52" s="63" t="s">
+      <c r="B52" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="C52" s="63" t="s">
+      <c r="C52" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="D52" s="64" t="s">
+      <c r="D52" s="69" t="s">
         <v>190</v>
       </c>
-      <c r="E52" s="67" t="s">
+      <c r="E52" s="64" t="s">
         <v>204</v>
       </c>
-      <c r="F52" s="67" t="s">
+      <c r="F52" s="64" t="s">
         <v>25</v>
       </c>
       <c r="G52" s="24">
@@ -4801,10 +5067,10 @@
       <c r="Z52" s="56"/>
     </row>
     <row r="53" spans="1:26" ht="54.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="62"/>
-      <c r="B53" s="62"/>
-      <c r="C53" s="62"/>
-      <c r="D53" s="62"/>
+      <c r="A53" s="61"/>
+      <c r="B53" s="61"/>
+      <c r="C53" s="61"/>
+      <c r="D53" s="61"/>
       <c r="E53" s="60"/>
       <c r="F53" s="60"/>
       <c r="G53" s="24">
@@ -4818,7 +5084,7 @@
       </c>
       <c r="J53" s="18"/>
       <c r="K53" s="18"/>
-      <c r="L53" s="62"/>
+      <c r="L53" s="61"/>
       <c r="M53" s="20"/>
       <c r="N53" s="21"/>
       <c r="O53" s="22" t="s">
@@ -4841,22 +5107,22 @@
       <c r="Z53" s="56"/>
     </row>
     <row r="54" spans="1:26" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="61" t="s">
+      <c r="A54" s="63" t="s">
         <v>207</v>
       </c>
-      <c r="B54" s="63" t="s">
+      <c r="B54" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="C54" s="63" t="s">
+      <c r="C54" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="D54" s="64" t="s">
+      <c r="D54" s="69" t="s">
         <v>190</v>
       </c>
-      <c r="E54" s="67" t="s">
+      <c r="E54" s="64" t="s">
         <v>208</v>
       </c>
-      <c r="F54" s="67" t="s">
+      <c r="F54" s="64" t="s">
         <v>25</v>
       </c>
       <c r="G54" s="24">
@@ -4895,10 +5161,10 @@
       <c r="Z54" s="56"/>
     </row>
     <row r="55" spans="1:26" ht="51" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="62"/>
-      <c r="B55" s="62"/>
-      <c r="C55" s="62"/>
-      <c r="D55" s="62"/>
+      <c r="A55" s="61"/>
+      <c r="B55" s="61"/>
+      <c r="C55" s="61"/>
+      <c r="D55" s="61"/>
       <c r="E55" s="60"/>
       <c r="F55" s="60"/>
       <c r="G55" s="24">
@@ -4912,7 +5178,7 @@
       </c>
       <c r="J55" s="18"/>
       <c r="K55" s="18"/>
-      <c r="L55" s="62"/>
+      <c r="L55" s="61"/>
       <c r="M55" s="20"/>
       <c r="N55" s="21"/>
       <c r="O55" s="22" t="s">
@@ -4935,22 +5201,22 @@
       <c r="Z55" s="56"/>
     </row>
     <row r="56" spans="1:26" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="61" t="s">
+      <c r="A56" s="63" t="s">
         <v>211</v>
       </c>
-      <c r="B56" s="63" t="s">
+      <c r="B56" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="C56" s="63" t="s">
+      <c r="C56" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="D56" s="64" t="s">
+      <c r="D56" s="69" t="s">
         <v>190</v>
       </c>
-      <c r="E56" s="67" t="s">
+      <c r="E56" s="64" t="s">
         <v>212</v>
       </c>
-      <c r="F56" s="67" t="s">
+      <c r="F56" s="64" t="s">
         <v>25</v>
       </c>
       <c r="G56" s="24">
@@ -4989,10 +5255,10 @@
       <c r="Z56" s="56"/>
     </row>
     <row r="57" spans="1:26" ht="51" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="62"/>
-      <c r="B57" s="62"/>
-      <c r="C57" s="62"/>
-      <c r="D57" s="62"/>
+      <c r="A57" s="61"/>
+      <c r="B57" s="61"/>
+      <c r="C57" s="61"/>
+      <c r="D57" s="61"/>
       <c r="E57" s="60"/>
       <c r="F57" s="60"/>
       <c r="G57" s="24">
@@ -5006,7 +5272,7 @@
       </c>
       <c r="J57" s="18"/>
       <c r="K57" s="18"/>
-      <c r="L57" s="62"/>
+      <c r="L57" s="61"/>
       <c r="M57" s="20"/>
       <c r="N57" s="21"/>
       <c r="O57" s="22" t="s">
@@ -5029,22 +5295,22 @@
       <c r="Z57" s="56"/>
     </row>
     <row r="58" spans="1:26" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="61" t="s">
+      <c r="A58" s="63" t="s">
         <v>216</v>
       </c>
-      <c r="B58" s="61" t="s">
+      <c r="B58" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="C58" s="61" t="s">
+      <c r="C58" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="D58" s="69" t="s">
+      <c r="D58" s="62" t="s">
         <v>217</v>
       </c>
-      <c r="E58" s="69" t="s">
+      <c r="E58" s="62" t="s">
         <v>218</v>
       </c>
-      <c r="F58" s="67" t="s">
+      <c r="F58" s="64" t="s">
         <v>25</v>
       </c>
       <c r="G58" s="40">
@@ -5059,7 +5325,7 @@
       <c r="J58" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="K58" s="70"/>
+      <c r="K58" s="65"/>
       <c r="L58" s="59"/>
       <c r="M58" s="20"/>
       <c r="N58" s="3"/>
@@ -5094,7 +5360,7 @@
       <c r="J59" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="K59" s="71"/>
+      <c r="K59" s="66"/>
       <c r="L59" s="60"/>
       <c r="M59" s="20"/>
       <c r="N59" s="3"/>
@@ -5129,7 +5395,7 @@
       <c r="J60" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="K60" s="71"/>
+      <c r="K60" s="66"/>
       <c r="L60" s="60"/>
       <c r="M60" s="20"/>
       <c r="N60" s="3"/>
@@ -5146,12 +5412,12 @@
       <c r="S60" s="22"/>
     </row>
     <row r="61" spans="1:26" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="62"/>
-      <c r="B61" s="62"/>
-      <c r="C61" s="62"/>
-      <c r="D61" s="62"/>
-      <c r="E61" s="62"/>
-      <c r="F61" s="62"/>
+      <c r="A61" s="61"/>
+      <c r="B61" s="61"/>
+      <c r="C61" s="61"/>
+      <c r="D61" s="61"/>
+      <c r="E61" s="61"/>
+      <c r="F61" s="61"/>
       <c r="G61" s="40">
         <v>4</v>
       </c>
@@ -5164,8 +5430,8 @@
       <c r="J61" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="K61" s="72"/>
-      <c r="L61" s="62"/>
+      <c r="K61" s="67"/>
+      <c r="L61" s="61"/>
       <c r="M61" s="20"/>
       <c r="N61" s="3"/>
       <c r="O61" s="22" t="s">
@@ -5181,22 +5447,22 @@
       <c r="S61" s="22"/>
     </row>
     <row r="62" spans="1:26" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="61" t="s">
+      <c r="A62" s="63" t="s">
         <v>226</v>
       </c>
-      <c r="B62" s="61" t="s">
+      <c r="B62" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="C62" s="61" t="s">
+      <c r="C62" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="D62" s="69" t="s">
+      <c r="D62" s="62" t="s">
         <v>227</v>
       </c>
-      <c r="E62" s="69" t="s">
+      <c r="E62" s="62" t="s">
         <v>228</v>
       </c>
-      <c r="F62" s="67" t="s">
+      <c r="F62" s="64" t="s">
         <v>25</v>
       </c>
       <c r="G62" s="40">
@@ -5211,7 +5477,7 @@
       <c r="J62" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="K62" s="70"/>
+      <c r="K62" s="65"/>
       <c r="L62" s="59"/>
       <c r="M62" s="20"/>
       <c r="N62" s="3"/>
@@ -5232,7 +5498,7 @@
       <c r="B63" s="60"/>
       <c r="C63" s="60"/>
       <c r="D63" s="60"/>
-      <c r="E63" s="62"/>
+      <c r="E63" s="61"/>
       <c r="F63" s="60"/>
       <c r="G63" s="40">
         <v>2</v>
@@ -5246,7 +5512,7 @@
       <c r="J63" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="K63" s="71"/>
+      <c r="K63" s="66"/>
       <c r="L63" s="60"/>
       <c r="M63" s="20"/>
       <c r="N63" s="3"/>
@@ -5267,7 +5533,7 @@
       <c r="B64" s="60"/>
       <c r="C64" s="60"/>
       <c r="D64" s="60"/>
-      <c r="E64" s="69" t="s">
+      <c r="E64" s="62" t="s">
         <v>233</v>
       </c>
       <c r="F64" s="60"/>
@@ -5283,7 +5549,7 @@
       <c r="J64" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="K64" s="71"/>
+      <c r="K64" s="66"/>
       <c r="L64" s="60"/>
       <c r="M64" s="20"/>
       <c r="N64" s="3"/>
@@ -5300,12 +5566,12 @@
       <c r="S64" s="22"/>
     </row>
     <row r="65" spans="1:19" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="62"/>
-      <c r="B65" s="62"/>
-      <c r="C65" s="62"/>
-      <c r="D65" s="62"/>
-      <c r="E65" s="62"/>
-      <c r="F65" s="62"/>
+      <c r="A65" s="61"/>
+      <c r="B65" s="61"/>
+      <c r="C65" s="61"/>
+      <c r="D65" s="61"/>
+      <c r="E65" s="61"/>
+      <c r="F65" s="61"/>
       <c r="G65" s="40">
         <v>4</v>
       </c>
@@ -5318,8 +5584,8 @@
       <c r="J65" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="K65" s="72"/>
-      <c r="L65" s="62"/>
+      <c r="K65" s="67"/>
+      <c r="L65" s="61"/>
       <c r="M65" s="20"/>
       <c r="N65" s="3"/>
       <c r="O65" s="22" t="s">
@@ -18433,15 +18699,77 @@
     </filterColumn>
   </autoFilter>
   <mergeCells count="95">
-    <mergeCell ref="L62:L65"/>
-    <mergeCell ref="E64:E65"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="C62:C65"/>
-    <mergeCell ref="D62:D65"/>
-    <mergeCell ref="E62:E63"/>
-    <mergeCell ref="F62:F65"/>
-    <mergeCell ref="K62:K65"/>
+    <mergeCell ref="L8:L10"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="L22:L27"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="D18:D21"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="L18:L21"/>
+    <mergeCell ref="A22:A27"/>
+    <mergeCell ref="B22:B27"/>
+    <mergeCell ref="C22:C27"/>
+    <mergeCell ref="D22:D27"/>
+    <mergeCell ref="F22:F27"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="L33:L34"/>
+    <mergeCell ref="F40:F42"/>
+    <mergeCell ref="L40:L42"/>
+    <mergeCell ref="A43:A45"/>
+    <mergeCell ref="B43:B45"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="D43:D45"/>
+    <mergeCell ref="E43:E45"/>
+    <mergeCell ref="F43:F45"/>
+    <mergeCell ref="L43:L45"/>
+    <mergeCell ref="A40:A42"/>
+    <mergeCell ref="B40:B42"/>
+    <mergeCell ref="C40:C42"/>
+    <mergeCell ref="D40:D42"/>
+    <mergeCell ref="E40:E42"/>
+    <mergeCell ref="L47:L48"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="D49:D50"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="L49:L50"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="D47:D48"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="L52:L53"/>
+    <mergeCell ref="A54:A55"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="E54:E55"/>
+    <mergeCell ref="F54:F55"/>
+    <mergeCell ref="L54:L55"/>
+    <mergeCell ref="A52:A53"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="F52:F53"/>
     <mergeCell ref="L56:L57"/>
     <mergeCell ref="A58:A61"/>
     <mergeCell ref="B58:B61"/>
@@ -18457,77 +18785,15 @@
     <mergeCell ref="E56:E57"/>
     <mergeCell ref="F56:F57"/>
     <mergeCell ref="K58:K61"/>
-    <mergeCell ref="L52:L53"/>
-    <mergeCell ref="A54:A55"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="E54:E55"/>
-    <mergeCell ref="F54:F55"/>
-    <mergeCell ref="L54:L55"/>
-    <mergeCell ref="A52:A53"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="F52:F53"/>
-    <mergeCell ref="L47:L48"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="L49:L50"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="D47:D48"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="F40:F42"/>
-    <mergeCell ref="L40:L42"/>
-    <mergeCell ref="A43:A45"/>
-    <mergeCell ref="B43:B45"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="D43:D45"/>
-    <mergeCell ref="E43:E45"/>
-    <mergeCell ref="F43:F45"/>
-    <mergeCell ref="L43:L45"/>
-    <mergeCell ref="A40:A42"/>
-    <mergeCell ref="B40:B42"/>
-    <mergeCell ref="C40:C42"/>
-    <mergeCell ref="D40:D42"/>
-    <mergeCell ref="E40:E42"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="L33:L34"/>
-    <mergeCell ref="L22:L27"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="C18:C21"/>
-    <mergeCell ref="D18:D21"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="L18:L21"/>
-    <mergeCell ref="A22:A27"/>
-    <mergeCell ref="B22:B27"/>
-    <mergeCell ref="C22:C27"/>
-    <mergeCell ref="D22:D27"/>
-    <mergeCell ref="F22:F27"/>
-    <mergeCell ref="L8:L10"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="L62:L65"/>
+    <mergeCell ref="E64:E65"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="C62:C65"/>
+    <mergeCell ref="D62:D65"/>
+    <mergeCell ref="E62:E63"/>
+    <mergeCell ref="F62:F65"/>
+    <mergeCell ref="K62:K65"/>
   </mergeCells>
   <conditionalFormatting sqref="I3:I6 I8:I10">
     <cfRule type="cellIs" dxfId="29" priority="1" stopIfTrue="1" operator="equal">

</xml_diff>